<commit_message>
feat(demo,ci): keyless demo mode with recorded Claude Opus 5.5 responses; full-pipeline CI
- Live golden set on anthropic/claude-opus-5-5 via the new structured-outputs adapter: 8/8 pass,
  injection fixture included. Those responses are committed as cassettes (examples/cassettes),
  so 'npm start -- evals/fixtures/01-*.json' works on a fresh clone with no API key.
- npm run eval:replay runs the whole pipeline over the golden set offline; CI now runs it, plus
  the Trigger.dev worker typecheck and every SQL proof against a fresh local Supabase.
- Demo rate card refreshed to 2026-10-v1, valid through 2026-12-31 (still invented); the sheet
  generator's validity is now fixed instead of now+90d, so the committed xlsx is reproducible.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rates/linkport-rate-sheet.xlsx
+++ b/rates/linkport-rate-sheet.xlsx
@@ -32,13 +32,13 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2026-06-v1</t>
+    <t>2026-10-v1</t>
   </si>
   <si>
     <t>Valid through</t>
   </si>
   <si>
-    <t>2026-06-30</t>
+    <t>2026-12-31</t>
   </si>
   <si>
     <t>Kind</t>

</xml_diff>